<commit_message>
Add Example Article Versions to 5.1 Sample IR Report (#284)
</commit_message>
<xml_diff>
--- a/source/_static/report/IR_sample_r51.xlsx
+++ b/source/_static/report/IR_sample_r51.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\siq\github\cop5\source\_static\report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{948CAE42-BD36-4F29-A5FD-FC103FB1F566}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{958DD62C-F45E-43D7-A998-B646EAF5E6AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4473" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4505" uniqueCount="286">
   <si>
     <t>Report_Name</t>
   </si>
@@ -883,6 +883,9 @@
   </si>
   <si>
     <t>P1:1234; ISNI:1234123412341234</t>
+  </si>
+  <si>
+    <t>VoR</t>
   </si>
 </sst>
 </file>
@@ -3107,6 +3110,9 @@
       <c r="F36" s="1" t="s">
         <v>97</v>
       </c>
+      <c r="G36" s="1" t="s">
+        <v>285</v>
+      </c>
       <c r="H36" s="1" t="s">
         <v>98</v>
       </c>
@@ -3208,6 +3214,9 @@
       <c r="F37" s="1" t="s">
         <v>97</v>
       </c>
+      <c r="G37" s="1" t="s">
+        <v>285</v>
+      </c>
       <c r="H37" s="1" t="s">
         <v>98</v>
       </c>
@@ -3309,6 +3318,9 @@
       <c r="F38" s="1" t="s">
         <v>97</v>
       </c>
+      <c r="G38" s="1" t="s">
+        <v>285</v>
+      </c>
       <c r="H38" s="1" t="s">
         <v>98</v>
       </c>
@@ -3410,6 +3422,9 @@
       <c r="F39" s="1" t="s">
         <v>97</v>
       </c>
+      <c r="G39" s="1" t="s">
+        <v>285</v>
+      </c>
       <c r="H39" s="1" t="s">
         <v>98</v>
       </c>
@@ -3511,6 +3526,9 @@
       <c r="F40" s="1" t="s">
         <v>97</v>
       </c>
+      <c r="G40" s="1" t="s">
+        <v>285</v>
+      </c>
       <c r="H40" s="1" t="s">
         <v>98</v>
       </c>
@@ -3612,6 +3630,9 @@
       <c r="F41" s="1" t="s">
         <v>97</v>
       </c>
+      <c r="G41" s="1" t="s">
+        <v>285</v>
+      </c>
       <c r="H41" s="1" t="s">
         <v>98</v>
       </c>
@@ -3713,6 +3734,9 @@
       <c r="F42" s="1" t="s">
         <v>97</v>
       </c>
+      <c r="G42" s="1" t="s">
+        <v>285</v>
+      </c>
       <c r="H42" s="1" t="s">
         <v>98</v>
       </c>
@@ -3814,6 +3838,9 @@
       <c r="F43" s="1" t="s">
         <v>97</v>
       </c>
+      <c r="G43" s="1" t="s">
+        <v>285</v>
+      </c>
       <c r="H43" s="1" t="s">
         <v>98</v>
       </c>
@@ -3915,6 +3942,9 @@
       <c r="F44" s="1" t="s">
         <v>97</v>
       </c>
+      <c r="G44" s="1" t="s">
+        <v>285</v>
+      </c>
       <c r="H44" s="1" t="s">
         <v>98</v>
       </c>
@@ -4016,6 +4046,9 @@
       <c r="F45" s="1" t="s">
         <v>97</v>
       </c>
+      <c r="G45" s="1" t="s">
+        <v>285</v>
+      </c>
       <c r="H45" s="1" t="s">
         <v>98</v>
       </c>
@@ -4117,6 +4150,9 @@
       <c r="F46" s="1" t="s">
         <v>97</v>
       </c>
+      <c r="G46" s="1" t="s">
+        <v>285</v>
+      </c>
       <c r="H46" s="1" t="s">
         <v>98</v>
       </c>
@@ -4218,6 +4254,9 @@
       <c r="F47" s="1" t="s">
         <v>97</v>
       </c>
+      <c r="G47" s="1" t="s">
+        <v>285</v>
+      </c>
       <c r="H47" s="1" t="s">
         <v>98</v>
       </c>
@@ -11167,6 +11206,9 @@
       <c r="F124" s="1" t="s">
         <v>166</v>
       </c>
+      <c r="G124" s="1" t="s">
+        <v>285</v>
+      </c>
       <c r="H124" s="1" t="s">
         <v>167</v>
       </c>
@@ -11268,6 +11310,9 @@
       <c r="F125" s="1" t="s">
         <v>166</v>
       </c>
+      <c r="G125" s="1" t="s">
+        <v>285</v>
+      </c>
       <c r="H125" s="1" t="s">
         <v>167</v>
       </c>
@@ -11369,6 +11414,9 @@
       <c r="F126" s="1" t="s">
         <v>166</v>
       </c>
+      <c r="G126" s="1" t="s">
+        <v>285</v>
+      </c>
       <c r="H126" s="1" t="s">
         <v>167</v>
       </c>
@@ -11470,6 +11518,9 @@
       <c r="F127" s="1" t="s">
         <v>166</v>
       </c>
+      <c r="G127" s="1" t="s">
+        <v>285</v>
+      </c>
       <c r="H127" s="1" t="s">
         <v>167</v>
       </c>
@@ -11571,6 +11622,9 @@
       <c r="F128" s="1" t="s">
         <v>166</v>
       </c>
+      <c r="G128" s="1" t="s">
+        <v>285</v>
+      </c>
       <c r="H128" s="1" t="s">
         <v>167</v>
       </c>
@@ -11672,6 +11726,9 @@
       <c r="F129" s="1" t="s">
         <v>166</v>
       </c>
+      <c r="G129" s="1" t="s">
+        <v>285</v>
+      </c>
       <c r="H129" s="1" t="s">
         <v>167</v>
       </c>
@@ -11773,6 +11830,9 @@
       <c r="F130" s="1" t="s">
         <v>166</v>
       </c>
+      <c r="G130" s="1" t="s">
+        <v>285</v>
+      </c>
       <c r="H130" s="1" t="s">
         <v>167</v>
       </c>
@@ -11874,6 +11934,9 @@
       <c r="F131" s="1" t="s">
         <v>166</v>
       </c>
+      <c r="G131" s="1" t="s">
+        <v>285</v>
+      </c>
       <c r="H131" s="1" t="s">
         <v>167</v>
       </c>
@@ -11975,6 +12038,9 @@
       <c r="F132" s="1" t="s">
         <v>166</v>
       </c>
+      <c r="G132" s="1" t="s">
+        <v>285</v>
+      </c>
       <c r="H132" s="1" t="s">
         <v>167</v>
       </c>
@@ -12076,6 +12142,9 @@
       <c r="F133" s="1" t="s">
         <v>166</v>
       </c>
+      <c r="G133" s="1" t="s">
+        <v>285</v>
+      </c>
       <c r="H133" s="1" t="s">
         <v>167</v>
       </c>
@@ -12177,6 +12246,9 @@
       <c r="F134" s="1" t="s">
         <v>166</v>
       </c>
+      <c r="G134" s="1" t="s">
+        <v>285</v>
+      </c>
       <c r="H134" s="1" t="s">
         <v>167</v>
       </c>
@@ -12278,6 +12350,9 @@
       <c r="F135" s="1" t="s">
         <v>166</v>
       </c>
+      <c r="G135" s="1" t="s">
+        <v>285</v>
+      </c>
       <c r="H135" s="1" t="s">
         <v>167</v>
       </c>
@@ -12379,6 +12454,9 @@
       <c r="F136" s="1" t="s">
         <v>178</v>
       </c>
+      <c r="G136" s="1" t="s">
+        <v>285</v>
+      </c>
       <c r="H136" s="1" t="s">
         <v>179</v>
       </c>
@@ -12480,6 +12558,9 @@
       <c r="F137" s="1" t="s">
         <v>178</v>
       </c>
+      <c r="G137" s="1" t="s">
+        <v>285</v>
+      </c>
       <c r="H137" s="1" t="s">
         <v>179</v>
       </c>
@@ -12581,6 +12662,9 @@
       <c r="F138" s="1" t="s">
         <v>178</v>
       </c>
+      <c r="G138" s="1" t="s">
+        <v>285</v>
+      </c>
       <c r="H138" s="1" t="s">
         <v>179</v>
       </c>
@@ -12682,6 +12766,9 @@
       <c r="F139" s="1" t="s">
         <v>178</v>
       </c>
+      <c r="G139" s="1" t="s">
+        <v>285</v>
+      </c>
       <c r="H139" s="1" t="s">
         <v>179</v>
       </c>
@@ -12783,6 +12870,9 @@
       <c r="F140" s="1" t="s">
         <v>178</v>
       </c>
+      <c r="G140" s="1" t="s">
+        <v>285</v>
+      </c>
       <c r="H140" s="1" t="s">
         <v>179</v>
       </c>
@@ -12884,6 +12974,9 @@
       <c r="F141" s="1" t="s">
         <v>178</v>
       </c>
+      <c r="G141" s="1" t="s">
+        <v>285</v>
+      </c>
       <c r="H141" s="1" t="s">
         <v>179</v>
       </c>
@@ -12985,6 +13078,9 @@
       <c r="F142" s="1" t="s">
         <v>178</v>
       </c>
+      <c r="G142" s="1" t="s">
+        <v>285</v>
+      </c>
       <c r="H142" s="1" t="s">
         <v>179</v>
       </c>
@@ -13085,6 +13181,9 @@
       </c>
       <c r="F143" s="1" t="s">
         <v>178</v>
+      </c>
+      <c r="G143" s="1" t="s">
+        <v>285</v>
       </c>
       <c r="H143" s="1" t="s">
         <v>179</v>

</xml_diff>

<commit_message>
Remove Article_Version from sample IR Item 3 (Book)
</commit_message>
<xml_diff>
--- a/source/_static/report/IR_sample_r51.xlsx
+++ b/source/_static/report/IR_sample_r51.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\siq\github\cop5\source\_static\report\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\office\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{958DD62C-F45E-43D7-A998-B646EAF5E6AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85C141EC-EC88-47CE-AB68-53D3D45B6B57}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4505" uniqueCount="286">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4493" uniqueCount="286">
   <si>
     <t>Report_Name</t>
   </si>
@@ -929,7 +929,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1055,7 +1055,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AQ276"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.5703125" style="1" customWidth="1"/>
     <col min="2" max="2" width="16.7109375" style="1" customWidth="1"/>
@@ -3110,9 +3110,6 @@
       <c r="F36" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="G36" s="1" t="s">
-        <v>285</v>
-      </c>
       <c r="H36" s="1" t="s">
         <v>98</v>
       </c>
@@ -3214,9 +3211,6 @@
       <c r="F37" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="G37" s="1" t="s">
-        <v>285</v>
-      </c>
       <c r="H37" s="1" t="s">
         <v>98</v>
       </c>
@@ -3318,9 +3312,6 @@
       <c r="F38" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="G38" s="1" t="s">
-        <v>285</v>
-      </c>
       <c r="H38" s="1" t="s">
         <v>98</v>
       </c>
@@ -3422,9 +3413,6 @@
       <c r="F39" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="G39" s="1" t="s">
-        <v>285</v>
-      </c>
       <c r="H39" s="1" t="s">
         <v>98</v>
       </c>
@@ -3526,9 +3514,6 @@
       <c r="F40" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="G40" s="1" t="s">
-        <v>285</v>
-      </c>
       <c r="H40" s="1" t="s">
         <v>98</v>
       </c>
@@ -3630,9 +3615,6 @@
       <c r="F41" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="G41" s="1" t="s">
-        <v>285</v>
-      </c>
       <c r="H41" s="1" t="s">
         <v>98</v>
       </c>
@@ -3734,9 +3716,6 @@
       <c r="F42" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="G42" s="1" t="s">
-        <v>285</v>
-      </c>
       <c r="H42" s="1" t="s">
         <v>98</v>
       </c>
@@ -3838,9 +3817,6 @@
       <c r="F43" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="G43" s="1" t="s">
-        <v>285</v>
-      </c>
       <c r="H43" s="1" t="s">
         <v>98</v>
       </c>
@@ -3942,9 +3918,6 @@
       <c r="F44" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="G44" s="1" t="s">
-        <v>285</v>
-      </c>
       <c r="H44" s="1" t="s">
         <v>98</v>
       </c>
@@ -4046,9 +4019,6 @@
       <c r="F45" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="G45" s="1" t="s">
-        <v>285</v>
-      </c>
       <c r="H45" s="1" t="s">
         <v>98</v>
       </c>
@@ -4150,9 +4120,6 @@
       <c r="F46" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="G46" s="1" t="s">
-        <v>285</v>
-      </c>
       <c r="H46" s="1" t="s">
         <v>98</v>
       </c>
@@ -4253,9 +4220,6 @@
       </c>
       <c r="F47" s="1" t="s">
         <v>97</v>
-      </c>
-      <c r="G47" s="1" t="s">
-        <v>285</v>
       </c>
       <c r="H47" s="1" t="s">
         <v>98</v>

</xml_diff>